<commit_message>
Show submitted assessment records only
</commit_message>
<xml_diff>
--- a/student_records_template.xlsx
+++ b/student_records_template.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -453,10 +453,12 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="27" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,20 +504,30 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>star_level</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>stars</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>assessment_checked_at</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>submitted_status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>submitted_at</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>recommendation</t>
         </is>

</xml_diff>